<commit_message>
Training apps: time trained, editable session times, records and Merge with UKC
- Progress: minutes or hours trained this month, from every app that keeps time
- No Hangs and Rock Rings save how long they ran; Outside saves START to FINISH
- Gym Session, Tick List and Outside: start and finish can be put right on save
- Toasts for the hardest grade ever or of the last 30 days as a climb is ticked,
  and the longest session ever or of the last 30 days on FINISH
- Outside: "Merge with UKC" makes the session and that UKC day one - the
  session's time and note (UKC's if blank), the trad climbs of whichever has
  more. UKC's sport and boulders always count; unmerged, both are sessions

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/toasts.xlsx
+++ b/docs/toasts.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Toasts'!$A$1:$K$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Toasts'!$A$1:$K$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1350,58 +1350,278 @@
       <c r="K16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Gym Session, Tick List, Outside</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Wow, that's the highest grade we have seen you tick! Congrats.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>5.2 s</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>A tick harder than any saved of its kind - boulder, sport or trad - and than the session's own earlier ticks</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>common/records.js:61</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Sport counts the gym session, tick list and endurance together. Says nothing with nothing saved to beat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Gym Session, Tick List, Outside</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>That's the highest grade we have seen you tick this month! Congrats.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>5.2 s</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>As above, but only against the last 30 days, when it isn't the hardest ever</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>common/records.js:63</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Rolling 30 days, not the calendar month</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Gym Session, Lap Timer</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Wow, that's your longest session ever. You're getting strong!</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>5.2 s</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>On FINISH, the climbs (gym) or laps (lap timer) are more than in any saved session</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>common/records.js:73</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Not on a session reopened with the wrench, or a lap timer session typed in</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Gym Session, Lap Timer</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>That's your longest session this month. You're getting strong!</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>5.2 s</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>As above, on FINISH, but only against the last 30 days, when it isn't the longest ever</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>common/records.js:75</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Rolling 30 days, not the calendar month</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Endurance</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Last set - make it count</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>5.2 s</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Bottom</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>The final set of a session starts</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr"/>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>Idea</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>EXAMPLE - how a new idea looks. Edit or delete this row.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K17"/>
+  <autoFilter ref="A1:K21"/>
   <dataValidations count="5">
     <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Info,Warning,Action"</formula1>

</xml_diff>